<commit_message>
Authomatic update 16.12.2025 16:50:51,37
</commit_message>
<xml_diff>
--- a/files_to_edit/table_of_articles.xlsx
+++ b/files_to_edit/table_of_articles.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yotto\YandexDisk-gasilin@inion.ru\Developments\e-Library_to_IRBIS\files_to_edit\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD1F9807-8296-4A0D-9D2D-48A50C358DE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B81A23FB-55C1-4E5C-A85C-D5BEC6160107}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="115">
   <si>
     <t>author</t>
   </si>
@@ -85,10 +85,10 @@
     <t>review_output_data</t>
   </si>
   <si>
-    <t>Ленкевич, А.С. ; Латыпова, А.Р.</t>
-  </si>
-  <si>
-    <t>Деконструкция тела геймера: эксперименты разработчиков с интерфейсами и игровыми контроллерами</t>
+    <t>Kurtyılmaz, D.</t>
+  </si>
+  <si>
+    <t>В статье анализируется фильм «Пассажиры» как пример взаимодействия кинематографа с философской концепцией утопии. Критически рассматриваются противоречия, присущие стремлению к идеальному обществу.</t>
   </si>
   <si>
     <t>Galactica media: Journal of media studies</t>
@@ -97,307 +97,274 @@
     <t>2025</t>
   </si>
   <si>
-    <t>7</t>
-  </si>
-  <si>
-    <t>2</t>
-  </si>
-  <si>
-    <t>28-60</t>
-  </si>
-  <si>
-    <t>https://elibrary.ru/kqdpep</t>
-  </si>
-  <si>
-    <t>10.46539/gmd.v7i2.643</t>
+    <t>3</t>
+  </si>
+  <si>
+    <t>15-40</t>
+  </si>
+  <si>
+    <t>https://elibrary.ru/ioccfc</t>
+  </si>
+  <si>
+    <t>10.46539/gmd.v7i3.599</t>
   </si>
   <si>
     <t>2658-7734</t>
   </si>
   <si>
+    <t>английский</t>
+  </si>
+  <si>
+    <t>ООО НПО "Генезис.Фронтир.Наука"</t>
+  </si>
+  <si>
+    <t>online</t>
+  </si>
+  <si>
+    <t>2658-7734-e</t>
+  </si>
+  <si>
+    <t>Кучерова, А.В.</t>
+  </si>
+  <si>
+    <t>Длинный кадр в киноискусстве: философский анализ (на примере творчества А. А. Тарковского)</t>
+  </si>
+  <si>
+    <t>Автор анализирует философские подходы к интерпретации длинного кадра как эстетического инструмента в кинематографе А. А. Тарковского. Актуальность обусловлена интересом современного киноискусства к созерцательной эстетике.</t>
+  </si>
+  <si>
+    <t>41-69</t>
+  </si>
+  <si>
+    <t>https://elibrary.ru/vkvbod</t>
+  </si>
+  <si>
+    <t>10.46539/gmd.v7i3.672</t>
+  </si>
+  <si>
     <t>русский</t>
   </si>
   <si>
-    <t>ООО НПО "Генезис.Фронтир.Наука"</t>
-  </si>
-  <si>
-    <t>online</t>
-  </si>
-  <si>
-    <t>2658-7734-e</t>
-  </si>
-  <si>
-    <t>Скоморох, М.М.</t>
-  </si>
-  <si>
-    <t>If we were allowed to visit: прокрустов интерфейс и медиатравма</t>
-  </si>
-  <si>
-    <t>61-84</t>
-  </si>
-  <si>
-    <t>https://elibrary.ru/ncuqbi</t>
-  </si>
-  <si>
-    <t>10.46539/gmd.v7i2.644</t>
-  </si>
-  <si>
-    <t>Очеретяный, К.А.</t>
-  </si>
-  <si>
-    <t>Перверсивные интерфейсы: зияние, дрейф и пульсации как онтологические стили в компьютерных играх</t>
-  </si>
-  <si>
-    <t>85-102</t>
-  </si>
-  <si>
-    <t>https://elibrary.ru/wnqgpu</t>
-  </si>
-  <si>
-    <t>10.46539/gmd.v7i2.645</t>
-  </si>
-  <si>
-    <t>Кириченко, В.В.</t>
-  </si>
-  <si>
-    <t>Кринжплей и геймер-тело: сдвиг в нормативной грамматике игрового процесса</t>
-  </si>
-  <si>
-    <t>103-127</t>
-  </si>
-  <si>
-    <t>https://elibrary.ru/nnmqkc</t>
-  </si>
-  <si>
-    <t>10.46539/gmd.v7i2.646</t>
-  </si>
-  <si>
-    <t>Дыдров, А.А. ; Варламова, А.С.</t>
-  </si>
-  <si>
-    <t>A02.15.31</t>
-  </si>
-  <si>
-    <t>Философия лица и нейросетевые агенты</t>
-  </si>
-  <si>
-    <t>128-145</t>
-  </si>
-  <si>
-    <t>https://elibrary.ru/hepdsa</t>
-  </si>
-  <si>
-    <t>10.46539/gmd.v7i2.647</t>
-  </si>
-  <si>
-    <t>Мухина, С.Х.</t>
-  </si>
-  <si>
-    <t>A02.15.51</t>
-  </si>
-  <si>
-    <t>Интерфейс как практика себя, или каково это — быть живым в эпоху киборгов?</t>
-  </si>
-  <si>
-    <t>146-165</t>
-  </si>
-  <si>
-    <t>https://elibrary.ru/beaewe</t>
-  </si>
-  <si>
-    <t>10.46539/gmd.v7i2.648</t>
-  </si>
-  <si>
-    <t>Aliev, R.T.</t>
-  </si>
-  <si>
-    <t>Post-symbolic coloniality: the metasimulacrum of otherness in digital culture</t>
-  </si>
-  <si>
-    <t>166-186</t>
-  </si>
-  <si>
-    <t>https://elibrary.ru/btivei</t>
-  </si>
-  <si>
-    <t>10.46539/gmd.v7i2.649</t>
-  </si>
-  <si>
-    <t>английский</t>
-  </si>
-  <si>
-    <t>Маленко, М.Я.</t>
-  </si>
-  <si>
-    <t>187-208</t>
-  </si>
-  <si>
-    <t>https://elibrary.ru/shhdvw</t>
-  </si>
-  <si>
-    <t>10.46539/gmd.v7i2.650</t>
-  </si>
-  <si>
-    <t>Пеннер, Р.В.</t>
-  </si>
-  <si>
-    <t>В работе рассматриваются ключевые положения труда Бруно Латура «Политики природы. Как привить наукам демократию» и их развитие в идее эмпативного интерфейса. Методология включает герменевтический анализ текста Латура, сопоставление его идей с концепциями постструктуралистов, а также привлечение примеров из экосистем и цифровых технологий. Основной результат — идея эмпативного интерфейса как инструмента паритетного диалога между человеческими и нечеловеческими актантами.</t>
-  </si>
-  <si>
-    <t>209-219</t>
-  </si>
-  <si>
-    <t>https://elibrary.ru/qdkzyu</t>
-  </si>
-  <si>
-    <t>10.46539/gmd.v7i2.651</t>
-  </si>
-  <si>
-    <t>Азаров, К.В.</t>
-  </si>
-  <si>
-    <t>220-235</t>
-  </si>
-  <si>
-    <t>https://elibrary.ru/pbwkfw</t>
-  </si>
-  <si>
-    <t>10.46539/gmd.v7i2.652</t>
-  </si>
-  <si>
-    <t>Яковлева, Л.Ю.</t>
-  </si>
-  <si>
-    <t>Архитектура как интерфейс: связь, разрыв, поломка</t>
-  </si>
-  <si>
-    <t>236-252</t>
-  </si>
-  <si>
-    <t>https://elibrary.ru/adqwon</t>
-  </si>
-  <si>
-    <t>10.46539/gmd.v7i2.653</t>
-  </si>
-  <si>
-    <t>Kolesnikova, D.A.</t>
+    <t>Rotondi, A.</t>
+  </si>
+  <si>
+    <t>Медиа</t>
+  </si>
+  <si>
+    <t>Автор анализирует использование архивных материалов в документальном фильме Андрея Ужика «Автобиография Николае Чаушеску». Рассматривается подход режиссёра к созданию субъективного образа исторического персонажа.</t>
+  </si>
+  <si>
+    <t>70-95</t>
+  </si>
+  <si>
+    <t>https://elibrary.ru/gahpnt</t>
+  </si>
+  <si>
+    <t>10.46539/gmd.v7i3.576</t>
+  </si>
+  <si>
+    <t>Cengiz, M.F. ; Djellouli, M.</t>
+  </si>
+  <si>
+    <t>Спорт</t>
+  </si>
+  <si>
+    <t>В исследовании анализируется популярность турецких сериалов в Алжире и причины их предпочтения. Для сбора данных использовался метод опроса. Результаты показали, что более половины участников предпочитают турецкие сериалы.</t>
+  </si>
+  <si>
+    <t>96-121</t>
+  </si>
+  <si>
+    <t>https://elibrary.ru/typcnc</t>
+  </si>
+  <si>
+    <t>10.46539/gmd.v7i3.572</t>
+  </si>
+  <si>
+    <t>An, Yi. ; Lv, X.</t>
+  </si>
+  <si>
+    <t>Avatar identification and psychological ownership of virtual items: key drivers of post-purchase intention in online games</t>
+  </si>
+  <si>
+    <t>Идентификация, Виртуальное, Логика, Игра, Логицизм, Восприятие, Ощущение, Моделирование</t>
+  </si>
+  <si>
+    <t>Исследование посвящено анализу влияния идентификации аватара и психологической принадлежности на удовлетворённость потребителей, намерение совершить повторную покупку и «сарафанное радио» в контексте видеоигр. Использованы данные опроса 439 онлайн-игроков и моделирование структурными уравнениями.</t>
+  </si>
+  <si>
+    <t>122-154</t>
+  </si>
+  <si>
+    <t>https://elibrary.ru/owgtui</t>
+  </si>
+  <si>
+    <t>10.46539/gmd.v7i3.590</t>
+  </si>
+  <si>
+    <t>Game design patterns consolidation</t>
+  </si>
+  <si>
+    <t>Дизайн, Игра, Проектирование, Сравнительный анализ</t>
+  </si>
+  <si>
+    <t>В статье анализируются коллекции шаблонов для геймдизайна и выявляются их слабые стороны. Предлагаются методы для консолидации моделей на основе сравнительного анализа шести работ по формированию таких коллекций.</t>
+  </si>
+  <si>
+    <t>155-176</t>
+  </si>
+  <si>
+    <t>https://elibrary.ru/wjiuit</t>
+  </si>
+  <si>
+    <t>10.46539/gmd.v7i3.571</t>
+  </si>
+  <si>
+    <t>Popova, O.V. ; Grishin, N.V.</t>
+  </si>
+  <si>
+    <t>Сущность, Идентичность, Социальные сети, Большие данные, Города, Машинное обучение, Восприятие</t>
+  </si>
+  <si>
+    <t>В статье анализируется публичное обсуждение политики территориальной идентичности в социальных сетях на примере Пермской агломерации. Исследование основано на материалах из 25 групп ВКонтакте и использует технологии больших данных и машинного обучения.</t>
+  </si>
+  <si>
+    <t>177-190</t>
+  </si>
+  <si>
+    <t>https://elibrary.ru/canemt</t>
+  </si>
+  <si>
+    <t>10.46539/gmd.v7i3.593</t>
+  </si>
+  <si>
+    <t>Гладышев, В.И. ; Валеева, Э.М. ; Белова, Л.И.</t>
+  </si>
+  <si>
+    <t>Эпоха мессенджеров: как компенсаторное общение помогает преодолеть вызовы тотальной цифровизации (по материалам социологического исследования)</t>
+  </si>
+  <si>
+    <t>Цифровизация, Виртуальное, Одиночество, Социальные сети, Действительность, Цифровые технологии, Реальность, Личность, Глобальные проблемы, Разум</t>
+  </si>
+  <si>
+    <t>В статье анализируется влияние общения в мессенджерах и социальных сетях на коммуникативные потребности молодёжи. Исследование показывает, что виртуальное общение не деформирует потребности и не оказывает вредоносного влияния при разумном использовании.</t>
+  </si>
+  <si>
+    <t>191-214</t>
+  </si>
+  <si>
+    <t>https://elibrary.ru/pxodoq</t>
+  </si>
+  <si>
+    <t>10.46539/gmd.v7i3.592</t>
+  </si>
+  <si>
+    <t>Жуков, Д.С. ; Ловцов, В.А. ; Лямин, С.К.</t>
+  </si>
+  <si>
+    <t>Сообщества в социальных сетях: политическая мобилизация и эхо-камеры</t>
+  </si>
+  <si>
+    <t>Исследование посвящено анализу политизированных сообществ в социальной сети «ВКонтакте». Цель — отделить настоящую сетевую активность от имитационной. Применяются методы картирования сети, качественного кодирования и сетевого анализа.</t>
+  </si>
+  <si>
+    <t>215-241</t>
+  </si>
+  <si>
+    <t>https://elibrary.ru/dnoisq</t>
+  </si>
+  <si>
+    <t>10.46539/gmd.v7i3.573</t>
+  </si>
+  <si>
+    <t>Овчинников, А.В.</t>
+  </si>
+  <si>
+    <t>Войны</t>
+  </si>
+  <si>
+    <t>242-267</t>
+  </si>
+  <si>
+    <t>https://elibrary.ru/dfxzdq</t>
+  </si>
+  <si>
+    <t>10.46539/gmd.v7i3.585</t>
+  </si>
+  <si>
+    <t>В исследовании анализируется, как пять популярных турецких новостных сайтов представляют новости об искусственном интеллекте в X (Twitter). Цель работы — изучить влияние этих практик на восприятие аудитории.</t>
+  </si>
+  <si>
+    <t>268-306</t>
+  </si>
+  <si>
+    <t>https://elibrary.ru/rijxgd</t>
+  </si>
+  <si>
+    <t>10.46539/gmd.v7i3.578</t>
+  </si>
+  <si>
+    <t>Павлов, А.В.</t>
+  </si>
+  <si>
+    <t>В рецензии анализируется книга Шелли МакМурдо о первой киноадаптации «Кладбища домашних животных» Мэри Ламберт. Рассматриваются темы переоценки культурного статуса фильма, его жанровых особенностей и влияния на традиционные ценности.</t>
+  </si>
+  <si>
+    <t>307-318</t>
+  </si>
+  <si>
+    <t>https://elibrary.ru/yubdwd</t>
+  </si>
+  <si>
+    <t>10.46539/gmd.v7i3.675</t>
+  </si>
+  <si>
+    <t>Makhadi, A.M.</t>
+  </si>
+  <si>
+    <t>Yasa, H.</t>
+  </si>
+  <si>
+    <t>«Кладбище домашних животных» как культурная ценность</t>
+  </si>
+  <si>
+    <t>A02.61</t>
+  </si>
+  <si>
+    <t>A03</t>
+  </si>
+  <si>
+    <t>A04</t>
+  </si>
+  <si>
+    <t>«Войны памяти» местного значения и феномен «отмены» в медийных условиях «аккомодативной культуры» (кейс республики Татарстан)</t>
+  </si>
+  <si>
+    <t>Artificial intelligence and Internet journalism: presentation of Artificial Intelligence news to Internet and X (Twitter) users in Türkiye</t>
   </si>
   <si>
     <t>A02.41.41.71</t>
   </si>
   <si>
-    <t>From loom to code: rethinking interfaces through cyberfeminist practices</t>
-  </si>
-  <si>
-    <t>253-274</t>
-  </si>
-  <si>
-    <t>https://elibrary.ru/ndszdb</t>
-  </si>
-  <si>
-    <t>10.46539/gmd.v7i2.654</t>
-  </si>
-  <si>
-    <t>Бакуменко, Г.В. ; Бакланов, И.С. ; Бакланова, О.А.</t>
-  </si>
-  <si>
-    <t>A02.31.21</t>
-  </si>
-  <si>
-    <t>275-305</t>
-  </si>
-  <si>
-    <t>https://elibrary.ru/pwxpux</t>
-  </si>
-  <si>
-    <t>10.46539/gmd.v7i2.656</t>
-  </si>
-  <si>
-    <t>Деконструкция, Компьютерные игры, Дизайн, Искусственный интеллект, Цифровая культура</t>
-  </si>
-  <si>
-    <t>Особенности постдисциплинарного контроля над телом игрока в современной игровой индустрии с помощью технологий искусственного интеллекта и датчиков. Анализируется, как игровая фанатская культура деконструирует нормативный геймплей и ломает практики контроля.</t>
-  </si>
-  <si>
-    <t>Особенности восприятия цифрового искусства на примере игры If We Were Allowed To Visit. Исследуется феномен ремедиационного блока, связанный с разницей в скорости обработки информации компьютером и мозгом человека, а также концепция прокрустова интерфейса как способа отражения травмы, связанной с адаптацией к новым медиа.</t>
-  </si>
-  <si>
-    <t>Медиа, Компьютерные игры, Цифровая культура, Мышление, Искусственный интеллект</t>
-  </si>
-  <si>
-    <t>A02.41.41.61</t>
-  </si>
-  <si>
-    <t>Онтологические стили и особенности работы интерфейсов в контексте цифровой реальности. На примере компьютерных игр показано, как интерфейсы работают со стилями, такими как зияние, дрейф, пульсации, и как они легитимируют «отсутствие», создавая условия для альтернативных способов существования в (не)возможных мирах.</t>
-  </si>
-  <si>
-    <t>Эпистемология, Компьютерные игры, Логицизм, Онтология, Возможные миры, Виртуальная реальность, Дизайн</t>
-  </si>
-  <si>
-    <t>Компьютерные игры, Дизайн, Личность, Эстетика, Телесность, Компьютерныи игры, Виртуальная реальность</t>
-  </si>
-  <si>
-    <t>Социально-гуманитарные аспекты рефлексии нейросетевых технологий. Анализируется влияние этих технологий на социально-антропологические эффекты и гипотетические социальные риски. Особое внимание уделяется критике концепта «деантропологизации» и использованию метафоры «чёрного ящика» в контексте осмысления последствий нейросетевой экспансии, а также философии лица как возможного выхода из гносеологического тупика.</t>
-  </si>
-  <si>
-    <t>Нейросети, Дискурс, Рефлексия, Эпистемология, Социально-философский анализ, Искусственный интеллект</t>
-  </si>
-  <si>
-    <t>Рассматриваются современные цифровые технологии и связанные с ними жизненные практики, анализируется их влияние на повседневную жизнь и экзистенциальные установки человека. Обсуждается вопрос о возможности сохранения индивидуальности и экзистенциального опыта в условиях тотального влияния технологий.</t>
-  </si>
-  <si>
-    <t>Киборг, Животные, Ментальное, Интернет, Самость, Окружающая среда, Цифровые технологии, Экзистенция, Философия техники</t>
-  </si>
-  <si>
-    <t>Структурные трансформации различий в цифровой культуре через концепцию метасимулякра инаковости. Показано, как цифровые платформы интегрируют инаковость в архитектуру взаимодействия, нейтрализуя её разрушительную силу и превращая в предварительно отформатированный стимул.</t>
-  </si>
-  <si>
-    <t>Симулякр, Символ, Цифровая культура, Этика, Освобождение, Восприятие, Социальные сети</t>
-  </si>
-  <si>
-    <t>Автор рассматривает т.н. «этнологические видеоигры», основанные на реальном этнографическом и фольклорном материале, с акцентом на репрезентацию или симуляцию традиционного шаманства. Анализируется игра Never Alone с использованием людогерменевтического и структурно-семиотического методов, а также антропологических источников о шаманстве.</t>
-  </si>
-  <si>
-    <t>Герменевтика, Семиотика, Логика, Шаманизм, Праксис, Игра, Онтологический поворот, Мировосприятие, Структурализм</t>
-  </si>
-  <si>
-    <t>Герменевтика шаманcких видеоигр на примере «Kisima Inŋitchuŋa»</t>
-  </si>
-  <si>
-    <t>Медиа, Латур Б., Акторно-сетевая теория, Демократия, Философия науки, Постструктурализм, Цифровая культура</t>
-  </si>
-  <si>
-    <t>Построение коллективов, миров, интерфейсов: о перспективах политической экологии сквозь призму книги Бруно Латура «Политики природы. Как привить наукам демократию»</t>
-  </si>
-  <si>
-    <t>Автор проводит аналогии между дивинацией и интерфейсом, анализируя их взаимосвязь и инверсивность. В качестве примера исследуются модусы взаимодействия с дивинацией на материале европейской рецепции «И Цзин» от Лейбница до Л.Н. Толстого и Дж. Кейджа.</t>
-  </si>
-  <si>
-    <t>Толстой Л.Н., Лейбниц Г.В., Лао Цзы, Мышление, Игра, Ментальное, Деконструкция, Дизайн</t>
-  </si>
-  <si>
-    <t>Интерфейс как вывернутая дивинация: модусы «И Цзин», Л. Толстого и Дж. Кейджа</t>
-  </si>
-  <si>
-    <t>Функции архитектуры как интерфейса, связывающего жителей с культурой и пространством. Роль «умного дома» в объединении тела, воображения и технологий. Критический анализ основан на проблематике поломки как необходимого условия существования технологий и материальной среды обитания человека.</t>
-  </si>
-  <si>
-    <t>Медиа, Дизайн, Социокультурное, Телесность, Воображение, Новые технологии</t>
-  </si>
-  <si>
-    <t>Историческая преемственность между технологиями плетения, ранними вычислительными системами и современным дизайном интерфейсов. Интерфейсы переосмысляются как динамичные места сопротивления и альтернативного получения знаний, где взаимодействие воплощается с помощью экспериментов, телесных техник и художественной практики.</t>
-  </si>
-  <si>
-    <t>Медиа, Дизайн, Познание, Художественное творчество, Экспериментальная наука, Феминизм</t>
-  </si>
-  <si>
-    <t>Авторы анализируют свойства интерфейса в медиапространстве и обсуждают эвристический потенциал категории интерфейса в медиаисследованиях.</t>
-  </si>
-  <si>
-    <t>Медиа, Дизайн, Социокультурное, Философия культуры, Нейросети, Научная фантастика</t>
-  </si>
-  <si>
-    <t>Нейрометафора пользовательского интерфейса Уильяма Гибсона</t>
+    <t>Avalon in space, is dreaming of utopia no longer possible? A philosophical analysis of «Passengers»</t>
+  </si>
+  <si>
+    <t>Archive footages, re-enacting and (auto)biography in Andrei Ujică’s «The autobiography of Nicolae Ceaușescu»</t>
+  </si>
+  <si>
+    <t>Quantitative research on turkish TV series in Algeria: analytical study</t>
+  </si>
+  <si>
+    <t>Discussion of the directions of territorial identity policy by residents of the Perm agglomeration in the social network «VKontakte» online communities</t>
+  </si>
+  <si>
+    <t>Антиутопия, Киноискусство, Идеализм, Литература и философия, Мораль, Дискурс</t>
+  </si>
+  <si>
+    <t>Киноискусство, Восприятие, Темпоральность, Феноменология, Эстетика, Интерпретация, Арсеньев Н.С.</t>
+  </si>
+  <si>
+    <t>Животные, Традиционные ценности, Ужас, Числа, Женщины, Киноискусство</t>
   </si>
 </sst>
 </file>
@@ -755,7 +722,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:U14"/>
+  <dimension ref="A1:U13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="20.6640625" customWidth="1"/>
@@ -838,21 +805,21 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:21" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:21" ht="72" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>21</v>
       </c>
       <c r="B2" t="s">
-        <v>87</v>
+        <v>102</v>
       </c>
       <c r="C2" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>22</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>98</v>
       </c>
       <c r="F2" t="s">
         <v>23</v>
@@ -860,52 +827,52 @@
       <c r="H2" t="s">
         <v>24</v>
       </c>
-      <c r="I2" t="s">
+      <c r="I2">
+        <v>7</v>
+      </c>
+      <c r="J2" t="s">
         <v>25</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>26</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="L2" s="2" t="s">
+      <c r="M2" t="s">
         <v>28</v>
       </c>
-      <c r="M2" t="s">
+      <c r="N2" t="s">
         <v>29</v>
       </c>
-      <c r="N2" t="s">
+      <c r="O2" t="s">
         <v>30</v>
       </c>
-      <c r="O2" t="s">
+      <c r="P2" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="P2" s="1" t="s">
+      <c r="Q2" t="s">
         <v>32</v>
       </c>
-      <c r="Q2" t="s">
+      <c r="R2" t="s">
         <v>33</v>
       </c>
-      <c r="R2" t="s">
+    </row>
+    <row r="3" spans="1:21" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="3" spans="1:21" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
+      <c r="B3" t="s">
+        <v>102</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="B3" t="s">
-        <v>101</v>
-      </c>
-      <c r="C3" s="1" t="s">
+      <c r="D3" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="E3" s="1" t="s">
         <v>36</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>99</v>
       </c>
       <c r="F3" t="s">
         <v>23</v>
@@ -913,11 +880,11 @@
       <c r="H3" t="s">
         <v>24</v>
       </c>
-      <c r="I3" t="s">
+      <c r="I3">
+        <v>7</v>
+      </c>
+      <c r="J3" t="s">
         <v>25</v>
-      </c>
-      <c r="J3" t="s">
-        <v>26</v>
       </c>
       <c r="K3" t="s">
         <v>37</v>
@@ -929,36 +896,36 @@
         <v>39</v>
       </c>
       <c r="N3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="O3" t="s">
+        <v>40</v>
+      </c>
+      <c r="P3" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="P3" s="1" t="s">
+      <c r="Q3" t="s">
         <v>32</v>
       </c>
-      <c r="Q3" t="s">
+      <c r="R3" t="s">
         <v>33</v>
       </c>
-      <c r="R3" t="s">
-        <v>34</v>
-      </c>
     </row>
-    <row r="4" spans="1:21" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B4" t="s">
-        <v>51</v>
+        <v>103</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>41</v>
+        <v>109</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>103</v>
+        <v>42</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>102</v>
+        <v>43</v>
       </c>
       <c r="F4" t="s">
         <v>23</v>
@@ -966,103 +933,105 @@
       <c r="H4" t="s">
         <v>24</v>
       </c>
-      <c r="I4" t="s">
+      <c r="I4">
+        <v>7</v>
+      </c>
+      <c r="J4" t="s">
         <v>25</v>
       </c>
-      <c r="J4" t="s">
-        <v>26</v>
-      </c>
       <c r="K4" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="M4" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="N4" t="s">
+        <v>29</v>
+      </c>
+      <c r="O4" t="s">
         <v>30</v>
       </c>
-      <c r="O4" t="s">
+      <c r="P4" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="P4" s="1" t="s">
+      <c r="Q4" t="s">
         <v>32</v>
       </c>
-      <c r="Q4" t="s">
+      <c r="R4" t="s">
         <v>33</v>
       </c>
-      <c r="R4" t="s">
-        <v>34</v>
-      </c>
     </row>
-    <row r="5" spans="1:21" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B5" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>46</v>
+        <v>110</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="E5" s="1"/>
+        <v>48</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>49</v>
+      </c>
       <c r="F5" t="s">
         <v>23</v>
       </c>
       <c r="H5" t="s">
         <v>24</v>
       </c>
-      <c r="I5" t="s">
+      <c r="I5">
+        <v>7</v>
+      </c>
+      <c r="J5" t="s">
         <v>25</v>
       </c>
-      <c r="J5" t="s">
-        <v>26</v>
-      </c>
       <c r="K5" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="M5" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="N5" t="s">
+        <v>29</v>
+      </c>
+      <c r="O5" t="s">
         <v>30</v>
       </c>
-      <c r="O5" t="s">
+      <c r="P5" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="P5" s="1" t="s">
+      <c r="Q5" t="s">
         <v>32</v>
       </c>
-      <c r="Q5" t="s">
+      <c r="R5" t="s">
         <v>33</v>
       </c>
-      <c r="R5" t="s">
-        <v>34</v>
-      </c>
     </row>
-    <row r="6" spans="1:21" ht="100.8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:21" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="B6" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>106</v>
+        <v>55</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>105</v>
+        <v>56</v>
       </c>
       <c r="F6" t="s">
         <v>23</v>
@@ -1070,52 +1039,52 @@
       <c r="H6" t="s">
         <v>24</v>
       </c>
-      <c r="I6" t="s">
+      <c r="I6">
+        <v>7</v>
+      </c>
+      <c r="J6" t="s">
         <v>25</v>
       </c>
-      <c r="J6" t="s">
-        <v>26</v>
-      </c>
       <c r="K6" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="M6" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="N6" t="s">
+        <v>29</v>
+      </c>
+      <c r="O6" t="s">
         <v>30</v>
       </c>
-      <c r="O6" t="s">
+      <c r="P6" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="P6" s="1" t="s">
+      <c r="Q6" t="s">
         <v>32</v>
       </c>
-      <c r="Q6" t="s">
+      <c r="R6" t="s">
         <v>33</v>
       </c>
-      <c r="R6" t="s">
-        <v>34</v>
-      </c>
     </row>
-    <row r="7" spans="1:21" ht="115.2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>56</v>
+        <v>99</v>
       </c>
       <c r="B7" t="s">
-        <v>57</v>
+        <v>104</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>108</v>
+        <v>61</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>107</v>
+        <v>62</v>
       </c>
       <c r="F7" t="s">
         <v>23</v>
@@ -1123,52 +1092,52 @@
       <c r="H7" t="s">
         <v>24</v>
       </c>
-      <c r="I7" t="s">
+      <c r="I7">
+        <v>7</v>
+      </c>
+      <c r="J7" t="s">
         <v>25</v>
       </c>
-      <c r="J7" t="s">
-        <v>26</v>
-      </c>
       <c r="K7" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="M7" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="N7" t="s">
+        <v>29</v>
+      </c>
+      <c r="O7" t="s">
         <v>30</v>
       </c>
-      <c r="O7" t="s">
+      <c r="P7" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="P7" s="1" t="s">
+      <c r="Q7" t="s">
         <v>32</v>
       </c>
-      <c r="Q7" t="s">
+      <c r="R7" t="s">
         <v>33</v>
       </c>
-      <c r="R7" t="s">
-        <v>34</v>
-      </c>
     </row>
-    <row r="8" spans="1:21" ht="72" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:21" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="B8" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>63</v>
+        <v>111</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>110</v>
+        <v>67</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>109</v>
+        <v>68</v>
       </c>
       <c r="F8" t="s">
         <v>23</v>
@@ -1176,52 +1145,52 @@
       <c r="H8" t="s">
         <v>24</v>
       </c>
-      <c r="I8" t="s">
+      <c r="I8">
+        <v>7</v>
+      </c>
+      <c r="J8" t="s">
         <v>25</v>
       </c>
-      <c r="J8" t="s">
-        <v>26</v>
-      </c>
       <c r="K8" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="L8" s="2" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="M8" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="N8" t="s">
+        <v>29</v>
+      </c>
+      <c r="O8" t="s">
         <v>30</v>
       </c>
-      <c r="O8" t="s">
-        <v>67</v>
-      </c>
       <c r="P8" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q8" t="s">
         <v>32</v>
       </c>
-      <c r="Q8" t="s">
+      <c r="R8" t="s">
         <v>33</v>
       </c>
-      <c r="R8" t="s">
-        <v>34</v>
-      </c>
     </row>
-    <row r="9" spans="1:21" ht="100.8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:21" ht="144" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="B9" t="s">
-        <v>57</v>
+        <v>104</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>113</v>
+        <v>73</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>112</v>
+        <v>74</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>111</v>
+        <v>75</v>
       </c>
       <c r="F9" t="s">
         <v>23</v>
@@ -1229,52 +1198,52 @@
       <c r="H9" t="s">
         <v>24</v>
       </c>
-      <c r="I9" t="s">
+      <c r="I9">
+        <v>7</v>
+      </c>
+      <c r="J9" t="s">
         <v>25</v>
       </c>
-      <c r="J9" t="s">
-        <v>26</v>
-      </c>
       <c r="K9" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="L9" s="2" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="M9" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="N9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="O9" t="s">
+        <v>40</v>
+      </c>
+      <c r="P9" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="P9" s="1" t="s">
+      <c r="Q9" t="s">
         <v>32</v>
       </c>
-      <c r="Q9" t="s">
+      <c r="R9" t="s">
         <v>33</v>
       </c>
-      <c r="R9" t="s">
-        <v>34</v>
-      </c>
     </row>
-    <row r="10" spans="1:21" ht="100.8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="B10" t="s">
-        <v>93</v>
+        <v>104</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>115</v>
+        <v>80</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>114</v>
+        <v>42</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>73</v>
+        <v>81</v>
       </c>
       <c r="F10" t="s">
         <v>23</v>
@@ -1282,105 +1251,103 @@
       <c r="H10" t="s">
         <v>24</v>
       </c>
-      <c r="I10" t="s">
+      <c r="I10">
+        <v>7</v>
+      </c>
+      <c r="J10" t="s">
         <v>25</v>
       </c>
-      <c r="J10" t="s">
-        <v>26</v>
-      </c>
       <c r="K10" t="s">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="L10" s="2" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="M10" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="N10" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="O10" t="s">
+        <v>40</v>
+      </c>
+      <c r="P10" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="P10" s="1" t="s">
+      <c r="Q10" t="s">
         <v>32</v>
       </c>
-      <c r="Q10" t="s">
+      <c r="R10" t="s">
         <v>33</v>
       </c>
-      <c r="R10" t="s">
-        <v>34</v>
-      </c>
     </row>
-    <row r="11" spans="1:21" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="B11" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>118</v>
+        <v>105</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>116</v>
-      </c>
+        <v>86</v>
+      </c>
+      <c r="E11" s="1"/>
       <c r="F11" t="s">
         <v>23</v>
       </c>
       <c r="H11" t="s">
         <v>24</v>
       </c>
-      <c r="I11" t="s">
+      <c r="I11">
+        <v>7</v>
+      </c>
+      <c r="J11" t="s">
         <v>25</v>
       </c>
-      <c r="J11" t="s">
-        <v>26</v>
-      </c>
       <c r="K11" t="s">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="L11" s="2" t="s">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="M11" t="s">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="N11" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="O11" t="s">
+        <v>40</v>
+      </c>
+      <c r="P11" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="P11" s="1" t="s">
+      <c r="Q11" t="s">
         <v>32</v>
       </c>
-      <c r="Q11" t="s">
+      <c r="R11" t="s">
         <v>33</v>
       </c>
-      <c r="R11" t="s">
-        <v>34</v>
-      </c>
     </row>
-    <row r="12" spans="1:21" ht="72" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>81</v>
+        <v>100</v>
       </c>
       <c r="B12" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>82</v>
+        <v>106</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>120</v>
+        <v>42</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>119</v>
+        <v>90</v>
       </c>
       <c r="F12" t="s">
         <v>23</v>
@@ -1388,52 +1355,52 @@
       <c r="H12" t="s">
         <v>24</v>
       </c>
-      <c r="I12" t="s">
+      <c r="I12">
+        <v>7</v>
+      </c>
+      <c r="J12" t="s">
         <v>25</v>
       </c>
-      <c r="J12" t="s">
-        <v>26</v>
-      </c>
       <c r="K12" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="L12" s="2" t="s">
-        <v>84</v>
+        <v>92</v>
       </c>
       <c r="M12" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="N12" t="s">
+        <v>29</v>
+      </c>
+      <c r="O12" t="s">
         <v>30</v>
       </c>
-      <c r="O12" t="s">
+      <c r="P12" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="P12" s="1" t="s">
+      <c r="Q12" t="s">
         <v>32</v>
       </c>
-      <c r="Q12" t="s">
+      <c r="R12" t="s">
         <v>33</v>
       </c>
-      <c r="R12" t="s">
-        <v>34</v>
-      </c>
     </row>
-    <row r="13" spans="1:21" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:21" ht="72" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="B13" t="s">
-        <v>87</v>
+        <v>107</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>88</v>
+        <v>101</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>121</v>
+        <v>95</v>
       </c>
       <c r="F13" t="s">
         <v>23</v>
@@ -1441,88 +1408,35 @@
       <c r="H13" t="s">
         <v>24</v>
       </c>
-      <c r="I13" t="s">
+      <c r="I13">
+        <v>7</v>
+      </c>
+      <c r="J13" t="s">
         <v>25</v>
       </c>
-      <c r="J13" t="s">
-        <v>26</v>
-      </c>
       <c r="K13" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="L13" s="2" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="M13" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="N13" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="O13" t="s">
-        <v>67</v>
+        <v>40</v>
       </c>
       <c r="P13" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q13" t="s">
         <v>32</v>
       </c>
-      <c r="Q13" t="s">
+      <c r="R13" t="s">
         <v>33</v>
-      </c>
-      <c r="R13" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="14" spans="1:21" ht="72" x14ac:dyDescent="0.3">
-      <c r="A14" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="B14" t="s">
-        <v>87</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="E14" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="F14" t="s">
-        <v>23</v>
-      </c>
-      <c r="H14" t="s">
-        <v>24</v>
-      </c>
-      <c r="I14" t="s">
-        <v>25</v>
-      </c>
-      <c r="J14" t="s">
-        <v>26</v>
-      </c>
-      <c r="K14" t="s">
-        <v>94</v>
-      </c>
-      <c r="L14" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="M14" t="s">
-        <v>96</v>
-      </c>
-      <c r="N14" t="s">
-        <v>30</v>
-      </c>
-      <c r="O14" t="s">
-        <v>31</v>
-      </c>
-      <c r="P14" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="Q14" t="s">
-        <v>33</v>
-      </c>
-      <c r="R14" t="s">
-        <v>34</v>
       </c>
     </row>
   </sheetData>
@@ -1539,7 +1453,6 @@
     <hyperlink ref="L11" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
     <hyperlink ref="L12" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
     <hyperlink ref="L13" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
-    <hyperlink ref="L14" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>